<commit_message>
Update: multi-sheet registry with Набор1 and Набор2, updated README
</commit_message>
<xml_diff>
--- a/Реестр_клиентов.xlsx
+++ b/Реестр_клиентов.xlsx
@@ -2,13 +2,87 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Реестр" sheetId="1" r:id="rId1"/>
+    <sheet name="Набор1" sheetId="1" r:id="rId1"/>
+    <sheet name="Набор2" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+  <si>
+    <t>ФИО</t>
+  </si>
+  <si>
+    <t>Наименование клиента</t>
+  </si>
+  <si>
+    <t>ИНН</t>
+  </si>
+  <si>
+    <t>КПП</t>
+  </si>
+  <si>
+    <t>ОГРН</t>
+  </si>
+  <si>
+    <t>Дата ОГРН</t>
+  </si>
+  <si>
+    <t>Юрадрес клиента</t>
+  </si>
+  <si>
+    <t>Телефон клиента</t>
+  </si>
+  <si>
+    <t>Р/с</t>
+  </si>
+  <si>
+    <t>Банк</t>
+  </si>
+  <si>
+    <t>К/с</t>
+  </si>
+  <si>
+    <t>БИК</t>
+  </si>
+  <si>
+    <t>номер договора</t>
+  </si>
+  <si>
+    <t>дата договора</t>
+  </si>
+  <si>
+    <t>территория действия</t>
+  </si>
+  <si>
+    <t>срок действия с</t>
+  </si>
+  <si>
+    <t>срок действия по</t>
+  </si>
+  <si>
+    <t>Сумма_1</t>
+  </si>
+  <si>
+    <t>Сумма_2</t>
+  </si>
+  <si>
+    <t>Должность_подписанта_1</t>
+  </si>
+  <si>
+    <t>ФИО_подписанта_1</t>
+  </si>
+  <si>
+    <t>Должность_подписанта_2</t>
+  </si>
+  <si>
+    <t>ФИО_подписанта_2</t>
+  </si>
+  <si>
+    <t>Дата заполнения</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -270,77 +344,157 @@
       <v>14.08.2026</v>
     </c>
   </row>
-  <row r="4">
-    <c r="A4">
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <autoFilter ref="A1:X1"/>
+  <row r="1">
+    <c r="A1" t="s">
+      <v>0</v>
+    </c>
+    <c r="B1" t="s">
+      <v>1</v>
+    </c>
+    <c r="C1" t="s">
+      <v>2</v>
+    </c>
+    <c r="D1" t="s">
+      <v>3</v>
+    </c>
+    <c r="E1" t="s">
+      <v>4</v>
+    </c>
+    <c r="F1" t="s">
+      <v>5</v>
+    </c>
+    <c r="G1" t="s">
+      <v>6</v>
+    </c>
+    <c r="H1" t="s">
+      <v>7</v>
+    </c>
+    <c r="I1" t="s">
+      <v>8</v>
+    </c>
+    <c r="J1" t="s">
+      <v>9</v>
+    </c>
+    <c r="K1" t="s">
+      <v>10</v>
+    </c>
+    <c r="L1" t="s">
+      <v>11</v>
+    </c>
+    <c r="M1" t="s">
+      <v>12</v>
+    </c>
+    <c r="N1" t="s">
+      <v>13</v>
+    </c>
+    <c r="O1" t="s">
+      <v>14</v>
+    </c>
+    <c r="P1" t="s">
+      <v>15</v>
+    </c>
+    <c r="Q1" t="s">
+      <v>16</v>
+    </c>
+    <c r="R1" t="s">
+      <v>17</v>
+    </c>
+    <c r="S1" t="s">
+      <v>18</v>
+    </c>
+    <c r="T1" t="s">
+      <v>19</v>
+    </c>
+    <c r="U1" t="s">
+      <v>20</v>
+    </c>
+    <c r="V1" t="s">
+      <v>21</v>
+    </c>
+    <c r="W1" t="s">
+      <v>22</v>
+    </c>
+    <c r="X1" t="s">
+      <v>23</v>
+    </c>
+  </row>
+  <row r="2">
+    <c r="A2">
       <v>Сидоров Алексей Сергеевич</v>
     </c>
-    <c r="B4">
+    <c r="B2">
       <v>ООО «Альфа-Логистика»</v>
     </c>
-    <c r="C4">
+    <c r="C2">
       <v>7712345678</v>
     </c>
-    <c r="D4">
+    <c r="D2">
       <v>771201001</v>
     </c>
-    <c r="E4">
+    <c r="E2">
       <v>1157746123456</v>
     </c>
-    <c r="F4">
+    <c r="F2">
       <v>05.11.2015</v>
     </c>
-    <c r="G4">
+    <c r="G2">
       <v>123456, г. Москва, пр. Ленина, д. 10</v>
     </c>
-    <c r="H4">
+    <c r="H2">
       <v>+7 (499) 555-12-34</v>
     </c>
-    <c r="I4">
+    <c r="I2">
       <v>40702810500000098765</v>
     </c>
-    <c r="J4">
+    <c r="J2">
       <v>АО «Тинькофф»</v>
     </c>
-    <c r="K4">
+    <c r="K2">
       <v>30101810100000000450</v>
     </c>
-    <c r="L4">
+    <c r="L2">
       <v>044525777</v>
     </c>
-    <c r="M4">
+    <c r="M2">
       <v>ДГ-2025-003</v>
     </c>
-    <c r="N4">
-      <v>14.08.2026</v>
-    </c>
-    <c r="O4">
+    <c r="N2">
+      <v>14.08.2026</v>
+    </c>
+    <c r="O2">
       <v>ЦФО</v>
     </c>
-    <c r="P4">
-      <v>14.08.2026</v>
-    </c>
-    <c r="Q4">
+    <c r="P2">
+      <v>14.08.2026</v>
+    </c>
+    <c r="Q2">
       <v>13.08.2027</v>
     </c>
-    <c r="R4">
+    <c r="R2">
       <v>750000</v>
     </c>
-    <c r="S4">
+    <c r="S2">
       <v>787500</v>
     </c>
-    <c r="T4">
+    <c r="T2">
       <v>Генеральный директор</v>
     </c>
-    <c r="U4">
+    <c r="U2">
       <v>Сидоров А.С.</v>
     </c>
-    <c r="V4">
+    <c r="V2">
       <v>Экономист</v>
     </c>
-    <c r="W4">
+    <c r="W2">
       <v>Козлова Е.Д.</v>
     </c>
-    <c r="X4">
+    <c r="X2">
       <v>14.08.2026</v>
     </c>
   </row>

</xml_diff>